<commit_message>
Update property roles and restructure opening schedule into 120/90/60/45-day milestones.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/public/downloads/opening-checklist.xlsx
+++ b/docs/public/downloads/opening-checklist.xlsx
@@ -49,10 +49,10 @@
     <t>物件</t>
   </si>
   <si>
-    <t>物件の最終選定・承認を上位店から受けている</t>
-  </si>
-  <si>
-    <t>賃貸借契約を締結した（上位店確認後）</t>
+    <t>物件の最終選定を決定した（上位店のアドバイスを反映）</t>
+  </si>
+  <si>
+    <t>賃貸借契約を締結した（アドバイス反映後・開設者決定）</t>
   </si>
   <si>
     <t>内装・レイアウトが完了している</t>

</xml_diff>